<commit_message>
Update plan for Ramp-up-testing phase
</commit_message>
<xml_diff>
--- a/C/Project/ATM_Sim/Doc/Project timeline.xlsx
+++ b/C/Project/ATM_Sim/Doc/Project timeline.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hienm\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Jira project\Embedded\C\Project\ATM_Sim\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC28C30-23E8-4E42-BCDE-43E4BD4B851D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26013AA2-FE28-42F2-92B8-911427E01A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
   <si>
     <t>ATM Machine - (V - Model)</t>
   </si>
@@ -142,9 +142,6 @@
     <t>System design</t>
   </si>
   <si>
-    <t>Login / Transfer / Withdraw / Balance)</t>
-  </si>
-  <si>
     <t>Architecture design</t>
   </si>
   <si>
@@ -188,6 +185,15 @@
   </si>
   <si>
     <t>MS 4: Testing Complete</t>
+  </si>
+  <si>
+    <t>Ramp-up testing</t>
+  </si>
+  <si>
+    <t>Ramp-up-testing</t>
+  </si>
+  <si>
+    <t>16/10/2026</t>
   </si>
 </sst>
 </file>
@@ -305,7 +311,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -354,8 +360,14 @@
         <bgColor rgb="FF3A3F47"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB6D7A8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="21">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -615,11 +627,81 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -664,9 +746,6 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -699,31 +778,65 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -747,61 +860,55 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="9" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1145,7 +1252,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Y20"/>
+  <dimension ref="A1:Y21"/>
   <sheetFormatPr defaultColWidth="13.4609375" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.765625" customWidth="1"/>
@@ -1157,11 +1264,11 @@
   <sheetData>
     <row r="1" spans="1:25" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
-      <c r="B1" s="58" t="s">
+      <c r="B1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -1186,11 +1293,11 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A2" s="4"/>
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1263,7 +1370,7 @@
       <c r="H4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="31" t="s">
+      <c r="I4" s="7" t="s">
         <v>9</v>
       </c>
       <c r="J4" s="7" t="s">
@@ -1324,7 +1431,7 @@
       <c r="H5" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="32">
+      <c r="I5" s="16">
         <v>46152</v>
       </c>
       <c r="J5" s="16">
@@ -1371,406 +1478,421 @@
       <c r="Y5" s="10"/>
     </row>
     <row r="6" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="60">
+      <c r="A6" s="44">
         <v>1</v>
       </c>
-      <c r="B6" s="61" t="s">
+      <c r="B6" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="35" t="s">
+      <c r="E6" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="43"/>
-      <c r="G6" s="45" t="s">
-        <v>49</v>
-      </c>
-      <c r="H6" s="19"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
-      <c r="P6" s="19"/>
-      <c r="Q6" s="19"/>
-      <c r="R6" s="19"/>
-      <c r="S6" s="19"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="56" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
+      <c r="P6" s="18"/>
+      <c r="Q6" s="18"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="18"/>
       <c r="T6" s="11"/>
       <c r="U6" s="11"/>
-      <c r="V6" s="20"/>
+      <c r="V6" s="19"/>
       <c r="W6" s="9"/>
       <c r="X6" s="10"/>
       <c r="Y6" s="10"/>
     </row>
-    <row r="7" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="51"/>
-      <c r="B7" s="62"/>
-      <c r="C7" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21"/>
+    <row r="7" spans="1:25" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="63"/>
+      <c r="B7" s="64"/>
+      <c r="C7" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="55"/>
+      <c r="G7" s="57"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="20"/>
+      <c r="L7" s="20"/>
+      <c r="M7" s="20"/>
+      <c r="N7" s="20"/>
+      <c r="O7" s="20"/>
+      <c r="P7" s="20"/>
+      <c r="Q7" s="20"/>
+      <c r="R7" s="20"/>
+      <c r="S7" s="20"/>
       <c r="T7" s="11"/>
       <c r="U7" s="11"/>
-      <c r="V7" s="20"/>
+      <c r="V7" s="19"/>
       <c r="W7" s="9"/>
       <c r="X7" s="10"/>
       <c r="Y7" s="10"/>
     </row>
-    <row r="8" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="63">
-        <v>2</v>
-      </c>
-      <c r="B8" s="64" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" s="37" t="s">
+    <row r="8" spans="1:25" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="65"/>
+      <c r="B8" s="66"/>
+      <c r="C8" s="62" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="61" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="37">
+      <c r="E8" s="60">
         <v>46275</v>
       </c>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="47" t="s">
-        <v>40</v>
-      </c>
-      <c r="I8" s="40" t="s">
-        <v>51</v>
-      </c>
-      <c r="J8" s="21"/>
-      <c r="K8" s="21"/>
-      <c r="L8" s="21"/>
-      <c r="M8" s="21"/>
-      <c r="P8" s="21"/>
-      <c r="Q8" s="21"/>
-      <c r="R8" s="21"/>
-      <c r="S8" s="21"/>
+      <c r="F8" s="58"/>
+      <c r="G8" s="67"/>
+      <c r="H8" s="60" t="s">
+        <v>56</v>
+      </c>
+      <c r="I8" s="60"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
+      <c r="N8" s="59"/>
+      <c r="O8" s="59"/>
+      <c r="P8" s="20"/>
+      <c r="Q8" s="20"/>
+      <c r="R8" s="20"/>
+      <c r="S8" s="20"/>
       <c r="T8" s="11"/>
       <c r="U8" s="11"/>
-      <c r="V8" s="20"/>
+      <c r="V8" s="19"/>
       <c r="W8" s="9"/>
       <c r="X8" s="10"/>
       <c r="Y8" s="10"/>
     </row>
     <row r="9" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="51"/>
-      <c r="B9" s="62"/>
-      <c r="C9" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="48"/>
-      <c r="I9" s="41"/>
-      <c r="J9" s="21"/>
-      <c r="K9" s="21"/>
-      <c r="L9" s="21"/>
-      <c r="M9" s="21"/>
-      <c r="P9" s="21"/>
-      <c r="Q9" s="21"/>
-      <c r="R9" s="21"/>
-      <c r="S9" s="21"/>
+      <c r="A9" s="46">
+        <v>2</v>
+      </c>
+      <c r="B9" s="47" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="33" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="69"/>
+      <c r="I9" s="70"/>
+      <c r="J9" s="51" t="s">
+        <v>50</v>
+      </c>
+      <c r="K9" s="20"/>
+      <c r="L9" s="20"/>
+      <c r="M9" s="20"/>
+      <c r="N9" s="65"/>
+      <c r="O9" s="65"/>
+      <c r="P9" s="20"/>
+      <c r="Q9" s="20"/>
+      <c r="R9" s="20"/>
+      <c r="S9" s="20"/>
       <c r="T9" s="11"/>
       <c r="U9" s="11"/>
-      <c r="V9" s="20"/>
+      <c r="V9" s="19"/>
       <c r="W9" s="9"/>
       <c r="X9" s="10"/>
       <c r="Y9" s="10"/>
     </row>
     <row r="10" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="51"/>
-      <c r="B10" s="53"/>
-      <c r="C10" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="49"/>
-      <c r="I10" s="42"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="21"/>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="21"/>
-      <c r="R10" s="21"/>
-      <c r="S10" s="21"/>
+      <c r="A10" s="63"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="71"/>
+      <c r="I10" s="72"/>
+      <c r="J10" s="52"/>
+      <c r="K10" s="20"/>
+      <c r="L10" s="20"/>
+      <c r="M10" s="20"/>
+      <c r="N10" s="65"/>
+      <c r="O10" s="65"/>
+      <c r="P10" s="20"/>
+      <c r="Q10" s="20"/>
+      <c r="R10" s="20"/>
+      <c r="S10" s="20"/>
       <c r="T10" s="11"/>
       <c r="U10" s="11"/>
-      <c r="V10" s="20"/>
+      <c r="V10" s="19"/>
       <c r="W10" s="9"/>
       <c r="X10" s="10"/>
       <c r="Y10" s="10"/>
     </row>
     <row r="11" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="50">
-        <v>3</v>
-      </c>
-      <c r="B11" s="52" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="37">
-        <v>46366</v>
-      </c>
-      <c r="E11" s="37" t="s">
-        <v>52</v>
-      </c>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="54"/>
-      <c r="K11" s="54"/>
-      <c r="L11" s="56" t="s">
-        <v>53</v>
-      </c>
-      <c r="M11" s="21"/>
-      <c r="N11" s="11"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="21"/>
-      <c r="Q11" s="21"/>
-      <c r="R11" s="21"/>
-      <c r="S11" s="21"/>
+      <c r="A11" s="63"/>
+      <c r="B11" s="68"/>
+      <c r="C11" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="37"/>
+      <c r="E11" s="37"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="73"/>
+      <c r="I11" s="74"/>
+      <c r="J11" s="53"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="20"/>
+      <c r="M11" s="20"/>
+      <c r="N11" s="65"/>
+      <c r="O11" s="65"/>
+      <c r="P11" s="20"/>
+      <c r="Q11" s="20"/>
+      <c r="R11" s="20"/>
+      <c r="S11" s="20"/>
       <c r="T11" s="11"/>
       <c r="U11" s="11"/>
-      <c r="V11" s="20"/>
+      <c r="V11" s="19"/>
       <c r="W11" s="9"/>
       <c r="X11" s="10"/>
       <c r="Y11" s="10"/>
     </row>
     <row r="12" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="51"/>
-      <c r="B12" s="53"/>
-      <c r="C12" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="34"/>
-      <c r="J12" s="55"/>
-      <c r="K12" s="55"/>
-      <c r="L12" s="57"/>
-      <c r="M12" s="21"/>
+      <c r="A12" s="48">
+        <v>3</v>
+      </c>
+      <c r="B12" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="33">
+        <v>46366</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="40"/>
+      <c r="K12" s="40"/>
+      <c r="L12" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="M12" s="20"/>
       <c r="N12" s="11"/>
       <c r="O12" s="11"/>
-      <c r="P12" s="21"/>
-      <c r="Q12" s="21"/>
-      <c r="R12" s="21"/>
-      <c r="S12" s="21"/>
+      <c r="P12" s="20"/>
+      <c r="Q12" s="20"/>
+      <c r="R12" s="20"/>
+      <c r="S12" s="20"/>
       <c r="T12" s="11"/>
       <c r="U12" s="11"/>
-      <c r="V12" s="20"/>
+      <c r="V12" s="19"/>
       <c r="W12" s="9"/>
       <c r="X12" s="10"/>
       <c r="Y12" s="10"/>
     </row>
     <row r="13" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="65">
-        <v>4</v>
-      </c>
-      <c r="B13" s="66" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="37">
-        <v>46064</v>
-      </c>
-      <c r="E13" s="37">
-        <v>46214</v>
-      </c>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="34"/>
-      <c r="J13" s="21"/>
-      <c r="L13" s="21"/>
-      <c r="M13" s="27"/>
-      <c r="N13" s="29" t="s">
-        <v>55</v>
-      </c>
+      <c r="A13" s="63"/>
+      <c r="B13" s="68"/>
+      <c r="C13" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="41"/>
+      <c r="K13" s="41"/>
+      <c r="L13" s="39"/>
+      <c r="M13" s="20"/>
+      <c r="N13" s="11"/>
       <c r="O13" s="11"/>
-      <c r="P13" s="21"/>
-      <c r="Q13" s="21"/>
-      <c r="R13" s="21"/>
-      <c r="S13" s="21"/>
+      <c r="P13" s="20"/>
+      <c r="Q13" s="20"/>
+      <c r="R13" s="20"/>
+      <c r="S13" s="20"/>
       <c r="T13" s="11"/>
       <c r="U13" s="11"/>
-      <c r="V13" s="20"/>
-      <c r="W13" s="22"/>
+      <c r="V13" s="19"/>
+      <c r="W13" s="9"/>
       <c r="X13" s="10"/>
       <c r="Y13" s="10"/>
     </row>
     <row r="14" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="51"/>
-      <c r="B14" s="62"/>
-      <c r="C14" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="D14" s="67"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="34"/>
-      <c r="J14" s="21"/>
-      <c r="L14" s="21"/>
-      <c r="M14" s="28"/>
-      <c r="N14" s="30"/>
+      <c r="A14" s="30">
+        <v>4</v>
+      </c>
+      <c r="B14" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="33">
+        <v>46064</v>
+      </c>
+      <c r="E14" s="33">
+        <v>46214</v>
+      </c>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="20"/>
+      <c r="K14" s="65"/>
+      <c r="L14" s="20"/>
+      <c r="M14" s="26"/>
+      <c r="N14" s="28" t="s">
+        <v>54</v>
+      </c>
       <c r="O14" s="11"/>
-      <c r="P14" s="21"/>
-      <c r="Q14" s="21"/>
-      <c r="R14" s="21"/>
-      <c r="S14" s="21"/>
+      <c r="P14" s="20"/>
+      <c r="Q14" s="20"/>
+      <c r="R14" s="20"/>
+      <c r="S14" s="20"/>
       <c r="T14" s="11"/>
       <c r="U14" s="11"/>
-      <c r="V14" s="20"/>
-      <c r="W14" s="22"/>
+      <c r="V14" s="19"/>
+      <c r="W14" s="21"/>
       <c r="X14" s="10"/>
       <c r="Y14" s="10"/>
     </row>
     <row r="15" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="51"/>
-      <c r="B15" s="53"/>
-      <c r="C15" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="D15" s="36"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="34"/>
-      <c r="J15" s="21"/>
-      <c r="L15" s="21"/>
-      <c r="M15" s="28"/>
-      <c r="N15" s="30"/>
+      <c r="A15" s="63"/>
+      <c r="B15" s="64"/>
+      <c r="C15" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="34"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="65"/>
+      <c r="L15" s="20"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="29"/>
       <c r="O15" s="11"/>
-      <c r="P15" s="21"/>
-      <c r="Q15" s="21"/>
-      <c r="R15" s="21"/>
-      <c r="S15" s="21"/>
+      <c r="P15" s="20"/>
+      <c r="Q15" s="20"/>
+      <c r="R15" s="20"/>
+      <c r="S15" s="20"/>
       <c r="T15" s="11"/>
       <c r="U15" s="11"/>
-      <c r="V15" s="20"/>
-      <c r="W15" s="22"/>
+      <c r="V15" s="19"/>
+      <c r="W15" s="21"/>
       <c r="X15" s="10"/>
       <c r="Y15" s="10"/>
     </row>
     <row r="16" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="23"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="9"/>
-      <c r="Q16" s="9"/>
-      <c r="R16" s="9"/>
-      <c r="S16" s="9"/>
-      <c r="T16" s="9"/>
-      <c r="U16" s="9"/>
-      <c r="V16" s="9"/>
-      <c r="W16" s="9"/>
+      <c r="A16" s="63"/>
+      <c r="B16" s="68"/>
+      <c r="C16" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" s="35"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="65"/>
+      <c r="L16" s="20"/>
+      <c r="M16" s="27"/>
+      <c r="N16" s="29"/>
+      <c r="O16" s="11"/>
+      <c r="P16" s="20"/>
+      <c r="Q16" s="20"/>
+      <c r="R16" s="20"/>
+      <c r="S16" s="20"/>
+      <c r="T16" s="11"/>
+      <c r="U16" s="11"/>
+      <c r="V16" s="19"/>
+      <c r="W16" s="21"/>
       <c r="X16" s="10"/>
       <c r="Y16" s="10"/>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="A17" s="23"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="2"/>
-      <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
-      <c r="V17" s="2"/>
-      <c r="W17" s="2"/>
-      <c r="X17" s="3"/>
-      <c r="Y17" s="3"/>
+    <row r="17" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="22"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="9"/>
+      <c r="P17" s="9"/>
+      <c r="Q17" s="9"/>
+      <c r="R17" s="9"/>
+      <c r="S17" s="9"/>
+      <c r="T17" s="9"/>
+      <c r="U17" s="9"/>
+      <c r="V17" s="9"/>
+      <c r="W17" s="9"/>
+      <c r="X17" s="10"/>
+      <c r="Y17" s="10"/>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="3"/>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
-      <c r="R18" s="3"/>
-      <c r="S18" s="3"/>
-      <c r="T18" s="3"/>
-      <c r="U18" s="3"/>
-      <c r="V18" s="3"/>
-      <c r="W18" s="3"/>
+      <c r="A18" s="22"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+      <c r="T18" s="2"/>
+      <c r="U18" s="2"/>
+      <c r="V18" s="2"/>
+      <c r="W18" s="2"/>
       <c r="X18" s="3"/>
       <c r="Y18" s="3"/>
     </row>
@@ -1828,33 +1950,60 @@
       <c r="X20" s="3"/>
       <c r="Y20" s="3"/>
     </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
+      <c r="P21" s="3"/>
+      <c r="Q21" s="3"/>
+      <c r="R21" s="3"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
+      <c r="U21" s="3"/>
+      <c r="V21" s="3"/>
+      <c r="W21" s="3"/>
+      <c r="X21" s="3"/>
+      <c r="Y21" s="3"/>
+    </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="E9:E11"/>
+    <mergeCell ref="J9:J11"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="H9:I11"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="B9:B11"/>
     <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="I8:I10"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="E14:E16"/>
+    <mergeCell ref="L12:L13"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="J12:J13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated plan for system design
</commit_message>
<xml_diff>
--- a/C/Project/ATM_Sim/Doc/Project timeline.xlsx
+++ b/C/Project/ATM_Sim/Doc/Project timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Jira project\Embedded\C\Project\ATM_Sim\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26013AA2-FE28-42F2-92B8-911427E01A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A789C046-0724-461D-BBB7-0CAFEE7400A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
   <si>
     <t>ATM Machine - (V - Model)</t>
   </si>
@@ -193,7 +193,10 @@
     <t>Ramp-up-testing</t>
   </si>
   <si>
-    <t>16/10/2026</t>
+    <t>27/11/2026</t>
+  </si>
+  <si>
+    <t>30/11/2026</t>
   </si>
 </sst>
 </file>
@@ -367,7 +370,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -643,9 +646,60 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color rgb="FFCCCCCC"/>
       </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="medium">
         <color rgb="FFCCCCCC"/>
       </right>
@@ -658,50 +712,28 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
+      <left/>
       <right/>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top/>
-      <bottom/>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -766,69 +798,117 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -836,79 +916,43 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="9" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="9" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="9" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="9" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1264,11 +1308,11 @@
   <sheetData>
     <row r="1" spans="1:25" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -1293,11 +1337,11 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A2" s="4"/>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1478,23 +1522,23 @@
       <c r="Y5" s="10"/>
     </row>
     <row r="6" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="44">
+      <c r="A6" s="52">
         <v>1</v>
       </c>
-      <c r="B6" s="45" t="s">
+      <c r="B6" s="54" t="s">
         <v>34</v>
       </c>
       <c r="C6" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="50" t="s">
+      <c r="D6" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="50" t="s">
+      <c r="E6" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="54"/>
-      <c r="G6" s="56" t="s">
+      <c r="F6" s="39"/>
+      <c r="G6" s="41" t="s">
         <v>48</v>
       </c>
       <c r="H6" s="18"/>
@@ -1517,15 +1561,15 @@
       <c r="Y6" s="10"/>
     </row>
     <row r="7" spans="1:25" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="63"/>
-      <c r="B7" s="64"/>
+      <c r="A7" s="53"/>
+      <c r="B7" s="55"/>
       <c r="C7" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="55"/>
-      <c r="G7" s="57"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="42"/>
       <c r="H7" s="20"/>
       <c r="I7" s="20"/>
       <c r="J7" s="20"/>
@@ -1546,29 +1590,33 @@
       <c r="Y7" s="10"/>
     </row>
     <row r="8" spans="1:25" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="65"/>
-      <c r="B8" s="66"/>
-      <c r="C8" s="62" t="s">
+      <c r="A8" s="30"/>
+      <c r="B8" s="57" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="61" t="s">
+      <c r="D8" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="60">
+      <c r="E8" s="66">
         <v>46275</v>
       </c>
-      <c r="F8" s="58"/>
-      <c r="G8" s="67"/>
-      <c r="H8" s="60" t="s">
+      <c r="F8" s="26"/>
+      <c r="G8" s="31"/>
+      <c r="H8" s="67" t="s">
         <v>56</v>
       </c>
-      <c r="I8" s="60"/>
+      <c r="I8" s="68"/>
       <c r="J8" s="20"/>
       <c r="K8" s="20"/>
-      <c r="L8" s="20"/>
+      <c r="L8" s="70" t="s">
+        <v>50</v>
+      </c>
       <c r="M8" s="20"/>
-      <c r="N8" s="59"/>
-      <c r="O8" s="59"/>
+      <c r="N8" s="27"/>
+      <c r="O8" s="27"/>
       <c r="P8" s="20"/>
       <c r="Q8" s="20"/>
       <c r="R8" s="20"/>
@@ -1581,34 +1629,28 @@
       <c r="Y8" s="10"/>
     </row>
     <row r="9" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="46">
+      <c r="A9" s="56">
         <v>2</v>
       </c>
-      <c r="B9" s="47" t="s">
-        <v>39</v>
-      </c>
+      <c r="B9" s="57"/>
       <c r="C9" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="33" t="s">
-        <v>38</v>
-      </c>
-      <c r="E9" s="33" t="s">
-        <v>57</v>
+      <c r="D9" s="34">
+        <v>46366</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>51</v>
       </c>
       <c r="F9" s="20"/>
       <c r="G9" s="20"/>
-      <c r="H9" s="69"/>
-      <c r="I9" s="70"/>
-      <c r="J9" s="51" t="s">
-        <v>50</v>
-      </c>
-      <c r="K9" s="20"/>
-      <c r="L9" s="20"/>
+      <c r="J9" s="43"/>
+      <c r="K9" s="44"/>
+      <c r="L9" s="37"/>
       <c r="M9" s="20"/>
-      <c r="N9" s="65"/>
-      <c r="O9" s="65"/>
-      <c r="P9" s="20"/>
+      <c r="N9" s="20"/>
+      <c r="O9" s="20"/>
+      <c r="P9" s="30"/>
       <c r="Q9" s="20"/>
       <c r="R9" s="20"/>
       <c r="S9" s="20"/>
@@ -1620,24 +1662,22 @@
       <c r="Y9" s="10"/>
     </row>
     <row r="10" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="63"/>
-      <c r="B10" s="64"/>
+      <c r="A10" s="53"/>
+      <c r="B10" s="57"/>
       <c r="C10" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
       <c r="F10" s="20"/>
       <c r="G10" s="20"/>
-      <c r="H10" s="71"/>
-      <c r="I10" s="72"/>
-      <c r="J10" s="52"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="20"/>
+      <c r="J10" s="45"/>
+      <c r="K10" s="46"/>
+      <c r="L10" s="37"/>
       <c r="M10" s="20"/>
-      <c r="N10" s="65"/>
-      <c r="O10" s="65"/>
-      <c r="P10" s="20"/>
+      <c r="N10" s="20"/>
+      <c r="O10" s="20"/>
+      <c r="P10" s="30"/>
       <c r="Q10" s="20"/>
       <c r="R10" s="20"/>
       <c r="S10" s="20"/>
@@ -1649,24 +1689,22 @@
       <c r="Y10" s="10"/>
     </row>
     <row r="11" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="63"/>
-      <c r="B11" s="68"/>
+      <c r="A11" s="53"/>
+      <c r="B11" s="69"/>
       <c r="C11" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D11" s="37"/>
-      <c r="E11" s="37"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="36"/>
       <c r="F11" s="20"/>
       <c r="G11" s="20"/>
-      <c r="H11" s="73"/>
-      <c r="I11" s="74"/>
-      <c r="J11" s="53"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="20"/>
+      <c r="J11" s="47"/>
+      <c r="K11" s="48"/>
+      <c r="L11" s="38"/>
       <c r="M11" s="20"/>
-      <c r="N11" s="65"/>
-      <c r="O11" s="65"/>
-      <c r="P11" s="20"/>
+      <c r="N11" s="20"/>
+      <c r="O11" s="20"/>
+      <c r="P11" s="30"/>
       <c r="Q11" s="20"/>
       <c r="R11" s="20"/>
       <c r="S11" s="20"/>
@@ -1678,34 +1716,31 @@
       <c r="Y11" s="10"/>
     </row>
     <row r="12" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="48">
+      <c r="A12" s="64">
         <v>3</v>
       </c>
-      <c r="B12" s="49" t="s">
+      <c r="B12" s="65" t="s">
         <v>42</v>
       </c>
       <c r="C12" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="33">
-        <v>46366</v>
-      </c>
-      <c r="E12" s="33" t="s">
-        <v>51</v>
+      <c r="D12" s="34">
+        <v>46064</v>
+      </c>
+      <c r="E12" s="34" t="s">
+        <v>57</v>
       </c>
       <c r="F12" s="20"/>
       <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="40"/>
-      <c r="K12" s="40"/>
-      <c r="L12" s="38" t="s">
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+      <c r="M12" s="62"/>
+      <c r="N12" s="71"/>
+      <c r="O12" s="71"/>
+      <c r="P12" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="M12" s="20"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="20"/>
       <c r="Q12" s="20"/>
       <c r="R12" s="20"/>
       <c r="S12" s="20"/>
@@ -1717,24 +1752,21 @@
       <c r="Y12" s="10"/>
     </row>
     <row r="13" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="63"/>
-      <c r="B13" s="68"/>
+      <c r="A13" s="53"/>
+      <c r="B13" s="58"/>
       <c r="C13" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
       <c r="F13" s="20"/>
       <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
-      <c r="J13" s="41"/>
-      <c r="K13" s="41"/>
-      <c r="L13" s="39"/>
-      <c r="M13" s="20"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="20"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="20"/>
+      <c r="M13" s="63"/>
+      <c r="N13" s="72"/>
+      <c r="O13" s="72"/>
+      <c r="P13" s="74"/>
       <c r="Q13" s="20"/>
       <c r="R13" s="20"/>
       <c r="S13" s="20"/>
@@ -1746,36 +1778,32 @@
       <c r="Y13" s="10"/>
     </row>
     <row r="14" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="30">
+      <c r="A14" s="59">
         <v>4</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="60" t="s">
         <v>53</v>
       </c>
       <c r="C14" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="33">
-        <v>46064</v>
-      </c>
-      <c r="E14" s="33">
-        <v>46214</v>
+      <c r="D14" s="34" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" s="34">
+        <v>46338</v>
       </c>
       <c r="F14" s="20"/>
       <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
       <c r="J14" s="20"/>
-      <c r="K14" s="65"/>
+      <c r="K14" s="20"/>
       <c r="L14" s="20"/>
-      <c r="M14" s="26"/>
-      <c r="N14" s="28" t="s">
+      <c r="M14" s="30"/>
+      <c r="N14" s="20"/>
+      <c r="Q14" s="75"/>
+      <c r="R14" s="77" t="s">
         <v>54</v>
       </c>
-      <c r="O14" s="11"/>
-      <c r="P14" s="20"/>
-      <c r="Q14" s="20"/>
-      <c r="R14" s="20"/>
       <c r="S14" s="20"/>
       <c r="T14" s="11"/>
       <c r="U14" s="11"/>
@@ -1785,26 +1813,22 @@
       <c r="Y14" s="10"/>
     </row>
     <row r="15" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="63"/>
-      <c r="B15" s="64"/>
+      <c r="A15" s="53"/>
+      <c r="B15" s="55"/>
       <c r="C15" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="34"/>
-      <c r="E15" s="36"/>
+      <c r="D15" s="61"/>
+      <c r="E15" s="61"/>
       <c r="F15" s="20"/>
       <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
       <c r="J15" s="20"/>
-      <c r="K15" s="65"/>
+      <c r="K15" s="20"/>
       <c r="L15" s="20"/>
-      <c r="M15" s="27"/>
-      <c r="N15" s="29"/>
-      <c r="O15" s="11"/>
-      <c r="P15" s="20"/>
-      <c r="Q15" s="20"/>
-      <c r="R15" s="20"/>
+      <c r="M15" s="30"/>
+      <c r="N15" s="20"/>
+      <c r="Q15" s="76"/>
+      <c r="R15" s="78"/>
       <c r="S15" s="20"/>
       <c r="T15" s="11"/>
       <c r="U15" s="11"/>
@@ -1814,26 +1838,22 @@
       <c r="Y15" s="10"/>
     </row>
     <row r="16" spans="1:25" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="63"/>
-      <c r="B16" s="68"/>
+      <c r="A16" s="53"/>
+      <c r="B16" s="58"/>
       <c r="C16" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="35"/>
-      <c r="E16" s="37"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
       <c r="F16" s="20"/>
       <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
       <c r="J16" s="20"/>
-      <c r="K16" s="65"/>
+      <c r="K16" s="20"/>
       <c r="L16" s="20"/>
-      <c r="M16" s="27"/>
-      <c r="N16" s="29"/>
-      <c r="O16" s="11"/>
-      <c r="P16" s="20"/>
-      <c r="Q16" s="20"/>
-      <c r="R16" s="20"/>
+      <c r="M16" s="30"/>
+      <c r="N16" s="20"/>
+      <c r="Q16" s="76"/>
+      <c r="R16" s="78"/>
       <c r="S16" s="20"/>
       <c r="T16" s="11"/>
       <c r="U16" s="11"/>
@@ -1978,32 +1998,34 @@
       <c r="Y21" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="D9:D11"/>
-    <mergeCell ref="E9:E11"/>
-    <mergeCell ref="J9:J11"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="H9:I11"/>
+  <mergeCells count="27">
+    <mergeCell ref="Q14:Q16"/>
+    <mergeCell ref="R14:R16"/>
+    <mergeCell ref="M12:O13"/>
+    <mergeCell ref="P12:P13"/>
+    <mergeCell ref="L8:L11"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="E14:E16"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A9:A11"/>
-    <mergeCell ref="B9:B11"/>
     <mergeCell ref="D6:D7"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="L12:L13"/>
-    <mergeCell ref="K12:K13"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="E9:E11"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="J9:K11"/>
+    <mergeCell ref="H8:I8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>